<commit_message>
fix(converter): correct compound-unit gradient for affine unit tokens
Two bugs in compound-unit conversion (e.g. psig/ft → kPa/m):

1. Closure-over-loop-variable: bridge conversion functions captured
   the loop variables by reference, so all candidates used the last
   iteration's values. Fixed with a _make_conversion(f, t) factory.

2. Offset leak: token factors used the absolute conversion value f(1),
   which includes the affine offset for gauge/temperature units
   (1 psig ≈ 108 kPa absolute → 355 kPa/m instead of 22.62 kPa/m).
   Fixed by using the slope f(1) - f(0) instead.

Fixed bug in the GUI that prevented the conversion path to be displayed.
</commit_message>
<xml_diff>
--- a/tests/conversions_check.xlsx
+++ b/tests/conversions_check.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\unyts\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7E99D13-D002-46AC-BEE2-DEA0C6B4C2A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CC8A7CC-0F9C-490E-A22C-AEBF66E7F3D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="49176" yWindow="2160" windowWidth="36156" windowHeight="19512" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="45972" yWindow="-108" windowWidth="46296" windowHeight="25416" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$F$2256</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$F$2265</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4532" uniqueCount="1164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4596" uniqueCount="1177">
   <si>
     <t>source</t>
   </si>
@@ -3526,6 +3526,45 @@
   </si>
   <si>
     <t>sip</t>
+  </si>
+  <si>
+    <t>MPa/km</t>
+  </si>
+  <si>
+    <t>cm3/min/Pa</t>
+  </si>
+  <si>
+    <t>sm3/day/psi</t>
+  </si>
+  <si>
+    <t>scf/day/psi</t>
+  </si>
+  <si>
+    <t>cc/min/Torr</t>
+  </si>
+  <si>
+    <t>kPa/m</t>
+  </si>
+  <si>
+    <t>Pa/m</t>
+  </si>
+  <si>
+    <t>m/s</t>
+  </si>
+  <si>
+    <t>km/h</t>
+  </si>
+  <si>
+    <t>mD</t>
+  </si>
+  <si>
+    <t>scf/stb</t>
+  </si>
+  <si>
+    <t>sm3/sm3</t>
+  </si>
+  <si>
+    <t>psig/ft</t>
   </si>
 </sst>
 </file>
@@ -3885,12 +3924,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G2262"/>
+  <dimension ref="A1:G2294"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="42" customWidth="1"/>
     <col min="3" max="4" width="28.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="12.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
@@ -45318,10 +45357,10 @@
       </c>
       <c r="B1973" s="2" t="str">
         <f t="shared" si="31"/>
-        <v>SM3/DAY/ -&gt; sm3/day/bar</v>
+        <v>SM3/DAY/BAR -&gt; sm3/day/bar</v>
       </c>
       <c r="C1973" t="s">
-        <v>955</v>
+        <v>969</v>
       </c>
       <c r="D1973" t="s">
         <v>954</v>
@@ -45339,13 +45378,13 @@
       </c>
       <c r="B1974" s="2" t="str">
         <f t="shared" si="31"/>
-        <v>SM3/DAY/ -&gt; SM3/DAY/</v>
+        <v>SM3/DAY/BARA -&gt; SM3/DAY/BARSA</v>
       </c>
       <c r="C1974" t="s">
-        <v>955</v>
+        <v>973</v>
       </c>
       <c r="D1974" t="s">
-        <v>955</v>
+        <v>1091</v>
       </c>
       <c r="E1974">
         <v>1</v>
@@ -51378,7 +51417,6 @@
         <v>1000</v>
       </c>
       <c r="F2261">
-        <f>E2261/100000*9.80665</f>
         <v>9.8066500000000001E-2</v>
       </c>
     </row>
@@ -51403,8 +51441,680 @@
         <v>0.45138888888888801</v>
       </c>
     </row>
+    <row r="2263" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2263" s="1">
+        <v>2261</v>
+      </c>
+      <c r="B2263" s="2" t="str">
+        <f t="shared" ref="B2263:B2265" si="36">C2263&amp;" -&gt; " &amp;D2263</f>
+        <v>g/cc -&gt; MPa/km</v>
+      </c>
+      <c r="C2263" t="s">
+        <v>840</v>
+      </c>
+      <c r="D2263" t="s">
+        <v>1164</v>
+      </c>
+      <c r="E2263">
+        <v>1</v>
+      </c>
+      <c r="F2263">
+        <v>9.8066499998653907</v>
+      </c>
+    </row>
+    <row r="2264" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2264" s="1">
+        <v>2262</v>
+      </c>
+      <c r="B2264" s="2" t="str">
+        <f t="shared" si="36"/>
+        <v>cm3/min/Pa -&gt; sm3/day/psi</v>
+      </c>
+      <c r="C2264" t="s">
+        <v>1165</v>
+      </c>
+      <c r="D2264" t="s">
+        <v>1166</v>
+      </c>
+      <c r="E2264">
+        <v>1</v>
+      </c>
+      <c r="F2264">
+        <v>9.9284505020261609</v>
+      </c>
+    </row>
+    <row r="2265" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2265" s="1">
+        <v>2263</v>
+      </c>
+      <c r="B2265" s="2" t="str">
+        <f t="shared" si="36"/>
+        <v>cc/min/Torr -&gt; scf/day/psi</v>
+      </c>
+      <c r="C2265" t="s">
+        <v>1168</v>
+      </c>
+      <c r="D2265" t="s">
+        <v>1167</v>
+      </c>
+      <c r="E2265">
+        <v>1</v>
+      </c>
+      <c r="F2265">
+        <v>2.6298656758972201</v>
+      </c>
+    </row>
+    <row r="2266" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2266" s="1">
+        <v>2264</v>
+      </c>
+      <c r="B2266" s="2" t="str">
+        <f t="shared" ref="B2266:B2277" si="37">C2266&amp;" -&gt; " &amp;D2266</f>
+        <v>lb/ft3 -&gt; MPa/km</v>
+      </c>
+      <c r="C2266" t="s">
+        <v>843</v>
+      </c>
+      <c r="D2266" t="s">
+        <v>1164</v>
+      </c>
+      <c r="E2266">
+        <v>1</v>
+      </c>
+      <c r="F2266">
+        <v>0.15708746384408959</v>
+      </c>
+    </row>
+    <row r="2267" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2267" s="1">
+        <v>2265</v>
+      </c>
+      <c r="B2267" s="2" t="str">
+        <f t="shared" si="37"/>
+        <v>bara/m -&gt; MPa/km</v>
+      </c>
+      <c r="C2267" t="s">
+        <v>847</v>
+      </c>
+      <c r="D2267" t="s">
+        <v>1164</v>
+      </c>
+      <c r="E2267">
+        <v>1</v>
+      </c>
+      <c r="F2267">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="2268" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2268" s="1">
+        <v>2266</v>
+      </c>
+      <c r="B2268" s="2" t="str">
+        <f t="shared" si="37"/>
+        <v>kPa/m -&gt; Pa/m</v>
+      </c>
+      <c r="C2268" t="s">
+        <v>1169</v>
+      </c>
+      <c r="D2268" t="s">
+        <v>1170</v>
+      </c>
+      <c r="E2268">
+        <v>1</v>
+      </c>
+      <c r="F2268">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="2269" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2269" s="1">
+        <v>2267</v>
+      </c>
+      <c r="B2269" s="2" t="str">
+        <f t="shared" si="37"/>
+        <v>atmosphere -&gt; psia</v>
+      </c>
+      <c r="C2269" t="s">
+        <v>563</v>
+      </c>
+      <c r="D2269" t="s">
+        <v>554</v>
+      </c>
+      <c r="E2269">
+        <v>1</v>
+      </c>
+      <c r="F2269">
+        <v>14.695948775715101</v>
+      </c>
+    </row>
+    <row r="2270" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2270" s="1">
+        <v>2268</v>
+      </c>
+      <c r="B2270" s="2" t="str">
+        <f t="shared" si="37"/>
+        <v>psia -&gt; atmosphere</v>
+      </c>
+      <c r="C2270" t="s">
+        <v>554</v>
+      </c>
+      <c r="D2270" t="s">
+        <v>563</v>
+      </c>
+      <c r="E2270">
+        <v>14.695948775715101</v>
+      </c>
+      <c r="F2270">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2271" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2271" s="1">
+        <v>2269</v>
+      </c>
+      <c r="B2271" s="2" t="str">
+        <f t="shared" si="37"/>
+        <v>m/s -&gt; ft/sec</v>
+      </c>
+      <c r="C2271" t="s">
+        <v>1171</v>
+      </c>
+      <c r="D2271" t="s">
+        <v>1125</v>
+      </c>
+      <c r="E2271">
+        <v>1</v>
+      </c>
+      <c r="F2271">
+        <v>3.280839895013123</v>
+      </c>
+    </row>
+    <row r="2272" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2272" s="1">
+        <v>2270</v>
+      </c>
+      <c r="B2272" s="2" t="str">
+        <f t="shared" si="37"/>
+        <v>m/s -&gt; km/h</v>
+      </c>
+      <c r="C2272" t="s">
+        <v>1171</v>
+      </c>
+      <c r="D2272" t="s">
+        <v>1172</v>
+      </c>
+      <c r="E2272">
+        <v>1</v>
+      </c>
+      <c r="F2272">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="2273" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2273" s="1">
+        <v>2271</v>
+      </c>
+      <c r="B2273" s="2" t="str">
+        <f t="shared" si="37"/>
+        <v>Darcy -&gt; mD</v>
+      </c>
+      <c r="C2273" t="s">
+        <v>922</v>
+      </c>
+      <c r="D2273" t="s">
+        <v>1173</v>
+      </c>
+      <c r="E2273">
+        <v>1</v>
+      </c>
+      <c r="F2273">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="2274" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2274" s="1">
+        <v>2272</v>
+      </c>
+      <c r="B2274" s="2" t="str">
+        <f t="shared" si="37"/>
+        <v>mD -&gt; µm2</v>
+      </c>
+      <c r="C2274" t="s">
+        <v>1173</v>
+      </c>
+      <c r="D2274" t="s">
+        <v>229</v>
+      </c>
+      <c r="E2274">
+        <v>1</v>
+      </c>
+      <c r="F2274">
+        <v>9.869232999999999E-4</v>
+      </c>
+    </row>
+    <row r="2275" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2275" s="1">
+        <v>2273</v>
+      </c>
+      <c r="B2275" s="2" t="str">
+        <f t="shared" si="37"/>
+        <v>API -&gt; g/cc</v>
+      </c>
+      <c r="C2275" t="s">
+        <v>831</v>
+      </c>
+      <c r="D2275" t="s">
+        <v>840</v>
+      </c>
+      <c r="E2275">
+        <v>10</v>
+      </c>
+      <c r="F2275">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2276" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2276" s="1">
+        <v>2274</v>
+      </c>
+      <c r="B2276" s="2" t="str">
+        <f t="shared" si="37"/>
+        <v>API -&gt; g/cc</v>
+      </c>
+      <c r="C2276" t="s">
+        <v>831</v>
+      </c>
+      <c r="D2276" t="s">
+        <v>840</v>
+      </c>
+      <c r="E2276">
+        <v>60</v>
+      </c>
+      <c r="F2276">
+        <v>0.73890339425587404</v>
+      </c>
+    </row>
+    <row r="2277" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2277" s="1">
+        <v>2275</v>
+      </c>
+      <c r="B2277" s="2" t="str">
+        <f t="shared" si="37"/>
+        <v>scf/stb -&gt; sm3/sm3</v>
+      </c>
+      <c r="C2277" t="s">
+        <v>1174</v>
+      </c>
+      <c r="D2277" t="s">
+        <v>1175</v>
+      </c>
+      <c r="E2277">
+        <v>1</v>
+      </c>
+      <c r="F2277">
+        <v>0.17810769813021299</v>
+      </c>
+    </row>
+    <row r="2278" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2278" s="1">
+        <v>2276</v>
+      </c>
+      <c r="B2278" s="2" t="str">
+        <f t="shared" ref="B2278:B2294" si="38">C2278&amp;" -&gt; " &amp;D2278</f>
+        <v>Celsius -&gt; Fahrenheit</v>
+      </c>
+      <c r="C2278" t="s">
+        <v>105</v>
+      </c>
+      <c r="D2278" t="s">
+        <v>108</v>
+      </c>
+      <c r="E2278">
+        <v>0</v>
+      </c>
+      <c r="F2278">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2279" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2279" s="1">
+        <v>2277</v>
+      </c>
+      <c r="B2279" s="2" t="str">
+        <f t="shared" si="38"/>
+        <v>Celsius -&gt; Fahrenheit</v>
+      </c>
+      <c r="C2279" t="s">
+        <v>105</v>
+      </c>
+      <c r="D2279" t="s">
+        <v>108</v>
+      </c>
+      <c r="E2279">
+        <v>100</v>
+      </c>
+      <c r="F2279">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="2280" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2280" s="1">
+        <v>2278</v>
+      </c>
+      <c r="B2280" s="2" t="str">
+        <f t="shared" si="38"/>
+        <v>Celsius -&gt; Fahrenheit</v>
+      </c>
+      <c r="C2280" t="s">
+        <v>105</v>
+      </c>
+      <c r="D2280" t="s">
+        <v>108</v>
+      </c>
+      <c r="E2280">
+        <v>-40</v>
+      </c>
+      <c r="F2280">
+        <v>-40</v>
+      </c>
+    </row>
+    <row r="2281" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2281" s="1">
+        <v>2279</v>
+      </c>
+      <c r="B2281" s="2" t="str">
+        <f t="shared" si="38"/>
+        <v>Fahrenheit -&gt; Kelvin</v>
+      </c>
+      <c r="C2281" t="s">
+        <v>108</v>
+      </c>
+      <c r="D2281" t="s">
+        <v>114</v>
+      </c>
+      <c r="E2281">
+        <v>32</v>
+      </c>
+      <c r="F2281">
+        <v>273.14999999999998</v>
+      </c>
+    </row>
+    <row r="2282" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2282" s="1">
+        <v>2280</v>
+      </c>
+      <c r="B2282" s="2" t="str">
+        <f t="shared" si="38"/>
+        <v>Fahrenheit -&gt; Kelvin</v>
+      </c>
+      <c r="C2282" t="s">
+        <v>108</v>
+      </c>
+      <c r="D2282" t="s">
+        <v>114</v>
+      </c>
+      <c r="E2282">
+        <v>212</v>
+      </c>
+      <c r="F2282">
+        <v>373.15</v>
+      </c>
+    </row>
+    <row r="2283" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2283" s="1">
+        <v>2281</v>
+      </c>
+      <c r="B2283" s="2" t="str">
+        <f t="shared" si="38"/>
+        <v>Celsius -&gt; Rankine</v>
+      </c>
+      <c r="C2283" t="s">
+        <v>105</v>
+      </c>
+      <c r="D2283" t="s">
+        <v>111</v>
+      </c>
+      <c r="E2283">
+        <v>0</v>
+      </c>
+      <c r="F2283">
+        <v>491.67</v>
+      </c>
+    </row>
+    <row r="2284" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2284" s="1">
+        <v>2282</v>
+      </c>
+      <c r="B2284" s="2" t="str">
+        <f t="shared" si="38"/>
+        <v>Kelvin -&gt; Fahrenheit</v>
+      </c>
+      <c r="C2284" t="s">
+        <v>114</v>
+      </c>
+      <c r="D2284" t="s">
+        <v>108</v>
+      </c>
+      <c r="E2284">
+        <v>0</v>
+      </c>
+      <c r="F2284">
+        <v>-459.67</v>
+      </c>
+    </row>
+    <row r="2285" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2285" s="1">
+        <v>2283</v>
+      </c>
+      <c r="B2285" s="2" t="str">
+        <f t="shared" si="38"/>
+        <v>psi gauge -&gt; psia</v>
+      </c>
+      <c r="C2285" t="s">
+        <v>606</v>
+      </c>
+      <c r="D2285" t="s">
+        <v>554</v>
+      </c>
+      <c r="E2285">
+        <v>0</v>
+      </c>
+      <c r="F2285">
+        <v>14.6959</v>
+      </c>
+    </row>
+    <row r="2286" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2286" s="1">
+        <v>2284</v>
+      </c>
+      <c r="B2286" s="2" t="str">
+        <f t="shared" si="38"/>
+        <v>bar gauge -&gt; bara</v>
+      </c>
+      <c r="C2286" t="s">
+        <v>611</v>
+      </c>
+      <c r="D2286" t="s">
+        <v>559</v>
+      </c>
+      <c r="E2286">
+        <v>0</v>
+      </c>
+      <c r="F2286">
+        <v>1.01325</v>
+      </c>
+    </row>
+    <row r="2287" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2287" s="1">
+        <v>2285</v>
+      </c>
+      <c r="B2287" s="2" t="str">
+        <f t="shared" si="38"/>
+        <v>psi gauge -&gt; Pascal</v>
+      </c>
+      <c r="C2287" t="s">
+        <v>606</v>
+      </c>
+      <c r="D2287" t="s">
+        <v>566</v>
+      </c>
+      <c r="E2287">
+        <v>0</v>
+      </c>
+      <c r="F2287">
+        <v>101325</v>
+      </c>
+    </row>
+    <row r="2288" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2288" s="1">
+        <v>2286</v>
+      </c>
+      <c r="B2288" s="2" t="str">
+        <f t="shared" si="38"/>
+        <v>bar gauge -&gt; Pascal</v>
+      </c>
+      <c r="C2288" t="s">
+        <v>611</v>
+      </c>
+      <c r="D2288" t="s">
+        <v>566</v>
+      </c>
+      <c r="E2288">
+        <v>0</v>
+      </c>
+      <c r="F2288">
+        <v>101325</v>
+      </c>
+    </row>
+    <row r="2289" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2289" s="1">
+        <v>2287</v>
+      </c>
+      <c r="B2289" s="2" t="str">
+        <f t="shared" si="38"/>
+        <v>psig/ft -&gt; kPa/m</v>
+      </c>
+      <c r="C2289" t="s">
+        <v>1176</v>
+      </c>
+      <c r="D2289" t="s">
+        <v>1169</v>
+      </c>
+      <c r="E2289">
+        <v>1</v>
+      </c>
+      <c r="F2289">
+        <v>22.6206</v>
+      </c>
+    </row>
+    <row r="2290" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2290" s="1">
+        <v>2288</v>
+      </c>
+      <c r="B2290" s="2" t="str">
+        <f t="shared" si="38"/>
+        <v>psia/ft -&gt; kPa/m</v>
+      </c>
+      <c r="C2290" t="s">
+        <v>846</v>
+      </c>
+      <c r="D2290" t="s">
+        <v>1169</v>
+      </c>
+      <c r="E2290">
+        <v>1</v>
+      </c>
+      <c r="F2290">
+        <v>22.6206</v>
+      </c>
+    </row>
+    <row r="2291" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2291" s="1">
+        <v>2289</v>
+      </c>
+      <c r="B2291" s="2" t="str">
+        <f t="shared" si="38"/>
+        <v>psi/ft -&gt; kPa/m</v>
+      </c>
+      <c r="C2291" t="s">
+        <v>844</v>
+      </c>
+      <c r="D2291" t="s">
+        <v>1169</v>
+      </c>
+      <c r="E2291">
+        <v>1</v>
+      </c>
+      <c r="F2291">
+        <v>22.6206</v>
+      </c>
+    </row>
+    <row r="2292" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2292" s="1">
+        <v>2290</v>
+      </c>
+      <c r="B2292" s="2" t="str">
+        <f t="shared" si="38"/>
+        <v>psig/ft -&gt; MPa/km</v>
+      </c>
+      <c r="C2292" t="s">
+        <v>1176</v>
+      </c>
+      <c r="D2292" t="s">
+        <v>1164</v>
+      </c>
+      <c r="E2292">
+        <v>1</v>
+      </c>
+      <c r="F2292">
+        <v>22.6206</v>
+      </c>
+    </row>
+    <row r="2293" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2293" s="1">
+        <v>2291</v>
+      </c>
+      <c r="B2293" s="2" t="str">
+        <f t="shared" si="38"/>
+        <v>lb/ft3 -&gt; kPa/m</v>
+      </c>
+      <c r="C2293" t="s">
+        <v>843</v>
+      </c>
+      <c r="D2293" t="s">
+        <v>1169</v>
+      </c>
+      <c r="E2293">
+        <v>1</v>
+      </c>
+      <c r="F2293">
+        <v>0.157087</v>
+      </c>
+    </row>
+    <row r="2294" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2294" s="1">
+        <v>2292</v>
+      </c>
+      <c r="B2294" s="2" t="str">
+        <f t="shared" si="38"/>
+        <v>SgO -&gt; MPa/km</v>
+      </c>
+      <c r="C2294" t="s">
+        <v>833</v>
+      </c>
+      <c r="D2294" t="s">
+        <v>1164</v>
+      </c>
+      <c r="E2294">
+        <v>0.8</v>
+      </c>
+      <c r="F2294">
+        <v>7.845600000000001</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F2256" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:F2265" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>